<commit_message>
Fill importable workbook with real M1-M5 data + headcount
Replace the example rows in the 6-tab template's FP&A and Workforce tabs
with verified data from the source workbooks (M1=Jan 2026):
- 05 · FP&A → fpa_monthly: real GP target/actual + revenue M1-M6 per team
  (RM+Bank, S&F, Renew, ATA), M6 target only.
- 03 · Nhân sự → team_workforce: real headcount (total 59) +
  revenueContribution = recorded revenue M1-M5 per team.

Generator now derives $M values from the raw USD figures. Verified the
rebuilt workbook through the parser: headcount 59, Σ revenue M1-M5 = 2.1069 $M.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y9ZidjJJvinCo5moj6bLmq
</commit_message>
<xml_diff>
--- a/public/templates/OneIBC_BOD_Workbook.xlsx
+++ b/public/templates/OneIBC_BOD_Workbook.xlsx
@@ -1630,7 +1630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1839,35 +1839,19 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>45</v>
-      </c>
-      <c r="H3" t="n">
-        <v>82</v>
-      </c>
-      <c r="I3" t="n">
-        <v>12</v>
-      </c>
-      <c r="J3" t="n">
-        <v>95</v>
-      </c>
-      <c r="K3" t="n">
-        <v>4.3</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="M3" t="n">
-        <v>5</v>
-      </c>
-      <c r="N3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="O3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="P3" t="n">
-        <v>2.4</v>
-      </c>
+        <v>0.3338</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1887,41 +1871,25 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>support</t>
+          <t>revenue</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>60</v>
-      </c>
-      <c r="H4" t="n">
-        <v>88</v>
-      </c>
-      <c r="I4" t="n">
-        <v>15</v>
-      </c>
-      <c r="J4" t="n">
-        <v>80</v>
-      </c>
-      <c r="K4" t="n">
-        <v>4.8</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="M4" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="N4" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="O4" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="P4" t="n">
-        <v>2.9</v>
-      </c>
+        <v>0.2696</v>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1936,7 +1904,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ATA</t>
+          <t>Renew</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1947,40 +1915,24 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>25</v>
-      </c>
-      <c r="H5" t="n">
-        <v>84</v>
-      </c>
-      <c r="I5" t="n">
-        <v>18</v>
-      </c>
-      <c r="J5" t="n">
-        <v>70</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1.8</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="M5" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="N5" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" t="n">
-        <v>1.2</v>
-      </c>
+        <v>1.0493</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>initiative</t>
+          <t>team_workforce</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1990,41 +1942,35 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AI &amp; Automation Program</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>On Track</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>80</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>ATA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>9</v>
+      </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="n">
-        <v>3</v>
-      </c>
-      <c r="N6" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="O6" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="P6" t="n">
-        <v>2.25</v>
-      </c>
+      <c r="L6" t="n">
+        <v>0.4542</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>initiative</t>
+          <t>team_workforce</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2034,34 +1980,154 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Operational Efficiency</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Delayed</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>42</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>8</v>
+      </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="n">
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>team_workforce</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>jun</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>13</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>initiative</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>jun</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AI &amp; Automation Program</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>80</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>initiative</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>jun</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Operational Efficiency</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Delayed</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>42</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
         <v>2</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N10" t="n">
         <v>1.4</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O10" t="n">
         <v>0.84</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P10" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -2712,7 +2778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2863,7 +2929,7 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>fpa_monthly: tháng</t>
+          <t>fpa_monthly: tháng (M1=Jan 2026 … M6=Jun)</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
@@ -2974,13 +3040,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.0912</v>
+        <v>0.0992</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0343</v>
+        <v>0.0358</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0506</v>
+        <v>0.0525</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -3008,17 +3074,25 @@
           <t>RM + Bank</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.07539999999999999</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+        <v>0.0992</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0564</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.08459999999999999</v>
+      </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -3037,7 +3111,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fpa_forecast</t>
+          <t>fpa_monthly</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3050,27 +3124,25 @@
           <t>revenue</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.2262</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.1199</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0992</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.0833</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
@@ -3084,37 +3156,43 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>fpa_scenario</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RM + Bank</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0362</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0596</v>
+      </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>P50 · Base Case</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.587</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>1.0996</v>
-      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
@@ -3123,15 +3201,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>fpa_ci</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>RM + Bank</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0362</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0537</v>
+      </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -3142,16 +3238,921 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="n">
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RM + Bank</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>S&amp;F</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.0326</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0456</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>S&amp;F</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.0674</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0945</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>S&amp;F</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.0392</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0597</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>S&amp;F</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.0234</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.0302</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>S&amp;F</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.1045</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.0287</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.0396</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>S&amp;F</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Renew</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0.1759</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.2344</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.4139</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Renew</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1791</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.0925</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.1398</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Renew</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.0973</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.1118</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.1717</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Renew</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0.1433</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.0629</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0897</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Renew</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.2064</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.1392</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.2343</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Renew</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.1524</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ATA</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.0622</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.0736</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.1088</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ATA</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.0594</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.0493</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ATA</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.1015</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.1349</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ATA</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.0891</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.0446</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.06270000000000001</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ATA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.0898</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.08450000000000001</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>fpa_monthly</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ATA</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.08790000000000001</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>fpa_scenario</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>P50 · Base Case</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.587</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1.0996</v>
+      </c>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>fpa_ci</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="n">
         <v>0.629</v>
       </c>
-      <c r="S7" t="n">
+      <c r="S28" t="n">
         <v>0.851</v>
       </c>
-      <c r="T7" t="n">
+      <c r="T28" t="n">
         <v>0.555</v>
       </c>
-      <c r="U7" t="n">
+      <c r="U28" t="n">
         <v>0.925</v>
       </c>
     </row>

</xml_diff>